<commit_message>
ajustes com codex para estabilidade e velocidade na automação
</commit_message>
<xml_diff>
--- a/src/planilhas/dados_alunos.xlsx
+++ b/src/planilhas/dados_alunos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2efd89dfc1e65699/Documentos/sice_auto_visitas/src/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="399" documentId="13_ncr:1_{F5F8047C-DE32-4309-9E84-B3F7C0479108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC6F5F98-0A35-46C6-A705-07375CCAFC26}"/>
+  <xr:revisionPtr revIDLastSave="465" documentId="13_ncr:1_{F5F8047C-DE32-4309-9E84-B3F7C0479108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D5AD18A-23C2-4C65-9406-D0EDC5CECDDD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="66">
   <si>
     <t>Nome</t>
   </si>
@@ -229,6 +229,9 @@
   </si>
   <si>
     <t>RUAN PABLO DE ARAUJO DA SILVA</t>
+  </si>
+  <si>
+    <t>CONSORCIO &amp; CORRETAGEM DE SEGUROS PRIME LTDA</t>
   </si>
 </sst>
 </file>
@@ -321,7 +324,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -337,6 +340,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -369,7 +384,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -414,15 +429,31 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -684,10 +715,10 @@
       <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:12" ht="24" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="21">
+      <c r="B2" s="20">
         <v>3741720</v>
       </c>
       <c r="C2" s="19" t="s">
@@ -700,7 +731,7 @@
         <v>46279</v>
       </c>
       <c r="F2" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>8</v>
@@ -712,10 +743,10 @@
       <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:12" ht="24" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="21">
+      <c r="B3" s="20">
         <v>5257044</v>
       </c>
       <c r="C3" s="19" t="s">
@@ -728,7 +759,7 @@
         <v>46279</v>
       </c>
       <c r="F3" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>8</v>
@@ -740,10 +771,10 @@
       <c r="L3" s="1"/>
     </row>
     <row r="4" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="21">
+      <c r="B4" s="20">
         <v>3138903</v>
       </c>
       <c r="C4" s="18" t="s">
@@ -756,7 +787,7 @@
         <v>46267</v>
       </c>
       <c r="F4" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>8</v>
@@ -768,10 +799,10 @@
       <c r="L4" s="1"/>
     </row>
     <row r="5" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="20">
         <v>2622732</v>
       </c>
       <c r="C5" s="19" t="s">
@@ -784,7 +815,7 @@
         <v>46275</v>
       </c>
       <c r="F5" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>7</v>
@@ -796,10 +827,10 @@
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="20">
         <v>2546120</v>
       </c>
       <c r="C6" s="18" t="s">
@@ -812,7 +843,7 @@
         <v>46267</v>
       </c>
       <c r="F6" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>8</v>
@@ -824,10 +855,10 @@
       <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="20">
         <v>3389371</v>
       </c>
       <c r="C7" s="19" t="s">
@@ -840,7 +871,7 @@
         <v>46275</v>
       </c>
       <c r="F7" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>7</v>
@@ -852,10 +883,10 @@
       <c r="L7" s="1"/>
     </row>
     <row r="8" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="20">
         <v>5256919</v>
       </c>
       <c r="C8" s="19" t="s">
@@ -868,7 +899,7 @@
         <v>46275</v>
       </c>
       <c r="F8" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>7</v>
@@ -880,10 +911,10 @@
       <c r="L8" s="1"/>
     </row>
     <row r="9" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="20">
         <v>4985871</v>
       </c>
       <c r="C9" s="18" t="s">
@@ -896,7 +927,7 @@
         <v>46274</v>
       </c>
       <c r="F9" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>8</v>
@@ -908,10 +939,10 @@
       <c r="L9" s="1"/>
     </row>
     <row r="10" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="20">
         <v>2460499</v>
       </c>
       <c r="C10" s="19" t="s">
@@ -920,7 +951,9 @@
       <c r="D10" s="6">
         <v>40438</v>
       </c>
-      <c r="E10" s="7"/>
+      <c r="E10" s="7">
+        <v>46287</v>
+      </c>
       <c r="F10" s="8">
         <v>0</v>
       </c>
@@ -934,10 +967,10 @@
       <c r="L10" s="1"/>
     </row>
     <row r="11" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="21">
+      <c r="B11" s="20">
         <v>3483885</v>
       </c>
       <c r="C11" s="18" t="s">
@@ -950,7 +983,7 @@
         <v>46267</v>
       </c>
       <c r="F11" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>8</v>
@@ -962,10 +995,10 @@
       <c r="L11" s="1"/>
     </row>
     <row r="12" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="20">
         <v>2377615</v>
       </c>
       <c r="C12" s="18" t="s">
@@ -978,7 +1011,7 @@
         <v>46267</v>
       </c>
       <c r="F12" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>8</v>
@@ -990,10 +1023,10 @@
       <c r="L12" s="1"/>
     </row>
     <row r="13" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="20">
         <v>4451670</v>
       </c>
       <c r="C13" s="18" t="s">
@@ -1006,7 +1039,7 @@
         <v>46275</v>
       </c>
       <c r="F13" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>8</v>
@@ -1018,10 +1051,10 @@
       <c r="L13" s="1"/>
     </row>
     <row r="14" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="20">
         <v>2556156</v>
       </c>
       <c r="C14" s="19" t="s">
@@ -1034,7 +1067,7 @@
         <v>46275</v>
       </c>
       <c r="F14" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" s="6" t="s">
         <v>8</v>
@@ -1046,10 +1079,10 @@
       <c r="L14" s="1"/>
     </row>
     <row r="15" spans="1:12" ht="24" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="20">
         <v>4844208</v>
       </c>
       <c r="C15" s="19" t="s">
@@ -1062,7 +1095,7 @@
         <v>46275</v>
       </c>
       <c r="F15" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>7</v>
@@ -1074,10 +1107,10 @@
       <c r="L15" s="1"/>
     </row>
     <row r="16" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="20">
         <v>3582671</v>
       </c>
       <c r="C16" s="19" t="s">
@@ -1090,7 +1123,7 @@
         <v>46267</v>
       </c>
       <c r="F16" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>8</v>
@@ -1100,10 +1133,10 @@
       <c r="L16" s="5"/>
     </row>
     <row r="17" spans="1:7" ht="24" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="20">
         <v>3393820</v>
       </c>
       <c r="C17" s="19" t="s">
@@ -1116,17 +1149,17 @@
         <v>46275</v>
       </c>
       <c r="F17" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="B18" s="21">
+      <c r="B18" s="20">
         <v>2677350</v>
       </c>
       <c r="C18" s="19" t="s">
@@ -1139,17 +1172,17 @@
         <v>46275</v>
       </c>
       <c r="F18" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="21">
+      <c r="B19" s="20">
         <v>2583861</v>
       </c>
       <c r="C19" s="19" t="s">
@@ -1162,17 +1195,17 @@
         <v>46267</v>
       </c>
       <c r="F19" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="24" x14ac:dyDescent="0.25">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="21">
+      <c r="B20" s="20">
         <v>5256354</v>
       </c>
       <c r="C20" s="19" t="s">
@@ -1185,17 +1218,17 @@
         <v>46279</v>
       </c>
       <c r="F20" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="21">
+      <c r="B21" s="20">
         <v>5160874</v>
       </c>
       <c r="C21" s="19" t="s">
@@ -1208,17 +1241,17 @@
         <v>46279</v>
       </c>
       <c r="F21" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="21">
+      <c r="B22" s="20">
         <v>4927976</v>
       </c>
       <c r="C22" s="19" t="s">
@@ -1231,17 +1264,17 @@
         <v>46275</v>
       </c>
       <c r="F22" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="21">
+      <c r="B23" s="20">
         <v>3133871</v>
       </c>
       <c r="C23" s="19" t="s">
@@ -1254,17 +1287,17 @@
         <v>46279</v>
       </c>
       <c r="F23" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="21">
+      <c r="B24" s="20">
         <v>2469229</v>
       </c>
       <c r="C24" s="19" t="s">
@@ -1277,17 +1310,17 @@
         <v>46267</v>
       </c>
       <c r="F24" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="21">
+      <c r="B25" s="20">
         <v>5257024</v>
       </c>
       <c r="C25" s="19" t="s">
@@ -1300,17 +1333,17 @@
         <v>46267</v>
       </c>
       <c r="F25" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="21">
+      <c r="B26" s="20">
         <v>4232277</v>
       </c>
       <c r="C26" s="18" t="s">
@@ -1323,36 +1356,40 @@
         <v>46275</v>
       </c>
       <c r="F26" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A27" s="22" t="s">
+    <row r="27" spans="1:7" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A27" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="21">
+      <c r="B27" s="24">
         <v>2842290</v>
       </c>
-      <c r="C27" s="19" t="s">
+      <c r="C27" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="D27" s="6"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="8">
-        <v>1</v>
-      </c>
-      <c r="G27" s="6" t="s">
+      <c r="D27" s="25">
+        <v>36959</v>
+      </c>
+      <c r="E27" s="26">
+        <v>46287</v>
+      </c>
+      <c r="F27" s="27">
+        <v>0</v>
+      </c>
+      <c r="G27" s="25" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="21">
+      <c r="B28" s="20">
         <v>3161275</v>
       </c>
       <c r="C28" s="19" t="s">
@@ -1361,19 +1398,21 @@
       <c r="D28" s="6">
         <v>32986</v>
       </c>
-      <c r="E28" s="7"/>
+      <c r="E28" s="7">
+        <v>46287</v>
+      </c>
       <c r="F28" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="20">
         <v>2676088</v>
       </c>
       <c r="C29" s="19" t="s">
@@ -1382,57 +1421,67 @@
       <c r="D29" s="6">
         <v>29905</v>
       </c>
-      <c r="E29" s="7"/>
+      <c r="E29" s="7">
+        <v>46267</v>
+      </c>
       <c r="F29" s="8">
+        <v>0</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="36" x14ac:dyDescent="0.25">
+      <c r="A30" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="20">
+        <v>3480805</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" s="6">
+        <v>41517</v>
+      </c>
+      <c r="E30" s="7">
+        <v>46267</v>
+      </c>
+      <c r="F30" s="8">
+        <v>0</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A31" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="20">
+        <v>3277548</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="D31" s="25">
+        <v>40437</v>
+      </c>
+      <c r="E31" s="26">
+        <v>46275</v>
+      </c>
+      <c r="F31" s="27">
         <v>1</v>
       </c>
-      <c r="G29" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A30" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="21"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="8">
-        <v>0</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A31" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B31" s="21">
-        <v>2676088</v>
-      </c>
-      <c r="C31" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="D31" s="6">
-        <v>40437</v>
-      </c>
-      <c r="E31" s="7">
-        <v>46275</v>
-      </c>
-      <c r="F31" s="8">
-        <v>1</v>
-      </c>
-      <c r="G31" s="6" t="s">
+      <c r="G31" s="25" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="24" x14ac:dyDescent="0.25">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="B32" s="21">
+      <c r="B32" s="20">
         <v>2553990</v>
       </c>
       <c r="C32" s="19" t="s">
@@ -1445,17 +1494,17 @@
         <v>46275</v>
       </c>
       <c r="F32" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="24" x14ac:dyDescent="0.25">
-      <c r="A33" s="22" t="s">
+      <c r="A33" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="21">
+      <c r="B33" s="20">
         <v>4762128</v>
       </c>
       <c r="C33" s="19" t="s">
@@ -1468,17 +1517,17 @@
         <v>46279</v>
       </c>
       <c r="F33" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A34" s="22" t="s">
+      <c r="A34" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="21">
+      <c r="B34" s="20">
         <v>5257066</v>
       </c>
       <c r="C34" s="18" t="s">
@@ -1491,17 +1540,17 @@
         <v>46274</v>
       </c>
       <c r="F34" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="B35" s="21">
+      <c r="B35" s="20">
         <v>2686533</v>
       </c>
       <c r="C35" s="18" t="s">
@@ -1514,17 +1563,17 @@
         <v>46275</v>
       </c>
       <c r="F35" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A36" s="22" t="s">
+      <c r="A36" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="B36" s="21">
+      <c r="B36" s="20">
         <v>2465181</v>
       </c>
       <c r="C36" s="18" t="s">
@@ -1537,17 +1586,17 @@
         <v>46267</v>
       </c>
       <c r="F36" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A37" s="22" t="s">
+      <c r="A37" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="B37" s="21">
+      <c r="B37" s="20">
         <v>3499270</v>
       </c>
       <c r="C37" s="18" t="s">
@@ -1560,17 +1609,17 @@
         <v>46275</v>
       </c>
       <c r="F37" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A38" s="22" t="s">
+      <c r="A38" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B38" s="21">
+      <c r="B38" s="20">
         <v>3483855</v>
       </c>
       <c r="C38" s="19" t="s">
@@ -1588,10 +1637,10 @@
       </c>
     </row>
     <row r="39" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A39" s="20" t="s">
+      <c r="A39" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="B39" s="21">
+      <c r="B39" s="20">
         <v>2621989</v>
       </c>
       <c r="C39" s="19" t="s">
@@ -1600,7 +1649,9 @@
       <c r="D39" s="6">
         <v>40438</v>
       </c>
-      <c r="E39" s="7"/>
+      <c r="E39" s="7">
+        <v>46287</v>
+      </c>
       <c r="F39" s="8">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
ajustes: agora o login é manual e so depois das credenciais starta a automatização
</commit_message>
<xml_diff>
--- a/src/planilhas/dados_alunos.xlsx
+++ b/src/planilhas/dados_alunos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2efd89dfc1e65699/Documentos/sice_auto_visitas/src/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="465" documentId="13_ncr:1_{F5F8047C-DE32-4309-9E84-B3F7C0479108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D5AD18A-23C2-4C65-9406-D0EDC5CECDDD}"/>
+  <xr:revisionPtr revIDLastSave="547" documentId="13_ncr:1_{F5F8047C-DE32-4309-9E84-B3F7C0479108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22DDB200-13A2-4FCA-86EA-ABB337EB9029}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="68">
   <si>
     <t>Nome</t>
   </si>
@@ -232,6 +232,12 @@
   </si>
   <si>
     <t>CONSORCIO &amp; CORRETAGEM DE SEGUROS PRIME LTDA</t>
+  </si>
+  <si>
+    <t>COPY NORT INFORMÁTICA</t>
+  </si>
+  <si>
+    <t>Tianguá</t>
   </si>
 </sst>
 </file>
@@ -324,36 +330,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -384,7 +366,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -411,9 +393,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -423,37 +402,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -682,7 +639,7 @@
   <cols>
     <col min="1" max="1" width="31.88671875" style="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" style="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
@@ -697,7 +654,7 @@
       <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="11" t="s">
@@ -714,24 +671,24 @@
       </c>
       <c r="H1" s="11"/>
     </row>
-    <row r="2" spans="1:12" ht="24" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="20">
-        <v>3741720</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>24</v>
+    <row r="2" spans="1:12" ht="36" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="19">
+        <v>3480805</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>65</v>
       </c>
       <c r="D2" s="6">
-        <v>28209</v>
+        <v>41517</v>
       </c>
       <c r="E2" s="7">
-        <v>46279</v>
+        <v>46309</v>
       </c>
       <c r="F2" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>8</v>
@@ -742,24 +699,24 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
     </row>
-    <row r="3" spans="1:12" ht="24" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="B3" s="20">
-        <v>5257044</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>24</v>
+    <row r="3" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="19">
+        <v>4985871</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>11</v>
       </c>
       <c r="D3" s="6">
-        <v>28209</v>
+        <v>38700</v>
       </c>
       <c r="E3" s="7">
-        <v>46279</v>
+        <v>46309</v>
       </c>
       <c r="F3" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>8</v>
@@ -771,23 +728,23 @@
       <c r="L3" s="1"/>
     </row>
     <row r="4" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="20">
-        <v>3138903</v>
+      <c r="A4" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="19">
+        <v>5257066</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" s="6">
-        <v>40526</v>
+        <v>38700</v>
       </c>
       <c r="E4" s="7">
-        <v>46267</v>
+        <v>46309</v>
       </c>
       <c r="F4" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>8</v>
@@ -799,26 +756,26 @@
       <c r="L4" s="1"/>
     </row>
     <row r="5" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="20">
-        <v>2622732</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>26</v>
+      <c r="A5" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="19">
+        <v>2377615</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>15</v>
       </c>
       <c r="D5" s="6">
-        <v>37969</v>
+        <v>34238</v>
       </c>
       <c r="E5" s="7">
-        <v>46275</v>
+        <v>46309</v>
       </c>
       <c r="F5" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="1"/>
@@ -827,23 +784,23 @@
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="20">
-        <v>2546120</v>
+      <c r="A6" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="19">
+        <v>2465181</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6" s="6">
-        <v>30172</v>
+        <v>34238</v>
       </c>
       <c r="E6" s="7">
-        <v>46267</v>
+        <v>46309</v>
       </c>
       <c r="F6" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>8</v>
@@ -855,26 +812,26 @@
       <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="20">
-        <v>3389371</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>20</v>
+      <c r="A7" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="19">
+        <v>2583861</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>17</v>
       </c>
       <c r="D7" s="6">
-        <v>20622</v>
+        <v>25212</v>
       </c>
       <c r="E7" s="7">
-        <v>46275</v>
+        <v>46309</v>
       </c>
       <c r="F7" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="1"/>
@@ -883,26 +840,26 @@
       <c r="L7" s="1"/>
     </row>
     <row r="8" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="20">
-        <v>5256919</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>20</v>
+      <c r="A8" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="19">
+        <v>2469229</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>17</v>
       </c>
       <c r="D8" s="6">
-        <v>20622</v>
+        <v>25212</v>
       </c>
       <c r="E8" s="7">
-        <v>46275</v>
+        <v>46309</v>
       </c>
       <c r="F8" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="1"/>
@@ -911,23 +868,23 @@
       <c r="L8" s="1"/>
     </row>
     <row r="9" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="20">
-        <v>4985871</v>
+      <c r="A9" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="19">
+        <v>4451670</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D9" s="6">
-        <v>38700</v>
+        <v>38977</v>
       </c>
       <c r="E9" s="7">
-        <v>46274</v>
+        <v>46309</v>
       </c>
       <c r="F9" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>8</v>
@@ -939,23 +896,23 @@
       <c r="L9" s="1"/>
     </row>
     <row r="10" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="20">
-        <v>2460499</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>19</v>
+      <c r="A10" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="19">
+        <v>4232277</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>18</v>
       </c>
       <c r="D10" s="6">
-        <v>40438</v>
+        <v>38977</v>
       </c>
       <c r="E10" s="7">
-        <v>46287</v>
+        <v>46309</v>
       </c>
       <c r="F10" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>8</v>
@@ -967,51 +924,51 @@
       <c r="L10" s="1"/>
     </row>
     <row r="11" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="20">
-        <v>3483885</v>
+      <c r="A11" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="19">
+        <v>2686533</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D11" s="6">
-        <v>30172</v>
+        <v>38977</v>
       </c>
       <c r="E11" s="7">
-        <v>46267</v>
+        <v>46309</v>
       </c>
       <c r="F11" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="14"/>
+      <c r="H11" s="13"/>
       <c r="I11" s="1"/>
       <c r="J11" s="2"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
     </row>
     <row r="12" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="20">
-        <v>2377615</v>
+      <c r="A12" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="19">
+        <v>3499270</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D12" s="6">
-        <v>34238</v>
+        <v>38977</v>
       </c>
       <c r="E12" s="7">
-        <v>46267</v>
+        <v>46309</v>
       </c>
       <c r="F12" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>8</v>
@@ -1023,26 +980,26 @@
       <c r="L12" s="1"/>
     </row>
     <row r="13" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" s="20">
-        <v>4451670</v>
+      <c r="A13" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="19">
+        <v>3389371</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D13" s="6">
-        <v>38977</v>
+        <v>20622</v>
       </c>
       <c r="E13" s="7">
-        <v>46275</v>
+        <v>46309</v>
       </c>
       <c r="F13" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="1"/>
@@ -1051,26 +1008,26 @@
       <c r="L13" s="1"/>
     </row>
     <row r="14" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A14" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="20">
-        <v>2556156</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>22</v>
+      <c r="A14" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="19">
+        <v>5256919</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>20</v>
       </c>
       <c r="D14" s="6">
-        <v>40437</v>
+        <v>20622</v>
       </c>
       <c r="E14" s="7">
-        <v>46275</v>
+        <v>46309</v>
       </c>
       <c r="F14" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="1"/>
@@ -1078,24 +1035,24 @@
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
     </row>
-    <row r="15" spans="1:12" ht="24" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" s="20">
-        <v>4844208</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>23</v>
+    <row r="15" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="19">
+        <v>5160874</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>20</v>
       </c>
       <c r="D15" s="6">
-        <v>29116</v>
+        <v>20622</v>
       </c>
       <c r="E15" s="7">
-        <v>46275</v>
+        <v>46309</v>
       </c>
       <c r="F15" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>7</v>
@@ -1106,572 +1063,574 @@
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
     </row>
-    <row r="16" spans="1:12" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A16" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="B16" s="20">
-        <v>3582671</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>25</v>
+    <row r="16" spans="1:12" ht="24" x14ac:dyDescent="0.25">
+      <c r="A16" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="19">
+        <v>4844208</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="D16" s="6">
-        <v>29911</v>
+        <v>29116</v>
       </c>
       <c r="E16" s="7">
-        <v>46267</v>
+        <v>46309</v>
       </c>
       <c r="F16" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H16" s="4"/>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
     </row>
     <row r="17" spans="1:7" ht="24" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="19">
         <v>3393820</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="18" t="s">
         <v>23</v>
       </c>
       <c r="D17" s="6">
         <v>29116</v>
       </c>
       <c r="E17" s="7">
-        <v>46275</v>
+        <v>46309</v>
       </c>
       <c r="F17" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A18" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" s="20">
-        <v>2677350</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>26</v>
+    <row r="18" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A18" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="19">
+        <v>2553990</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="D18" s="6">
-        <v>37969</v>
+        <v>29116</v>
       </c>
       <c r="E18" s="7">
-        <v>46275</v>
+        <v>46309</v>
       </c>
       <c r="F18" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A19" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="B19" s="20">
-        <v>2583861</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>17</v>
+      <c r="A19" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="19">
+        <v>2622732</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>26</v>
       </c>
       <c r="D19" s="6">
-        <v>25212</v>
+        <v>37969</v>
       </c>
       <c r="E19" s="7">
-        <v>46267</v>
+        <v>46309</v>
       </c>
       <c r="F19" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="24" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="B20" s="20">
-        <v>5256354</v>
-      </c>
-      <c r="C20" s="19" t="s">
-        <v>24</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A20" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="19">
+        <v>2677350</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>26</v>
       </c>
       <c r="D20" s="6">
-        <v>28209</v>
+        <v>37969</v>
       </c>
       <c r="E20" s="7">
-        <v>46279</v>
+        <v>46309</v>
       </c>
       <c r="F20" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A21" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="B21" s="20">
-        <v>5160874</v>
-      </c>
-      <c r="C21" s="19" t="s">
-        <v>20</v>
+      <c r="A21" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="19">
+        <v>3483855</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>9</v>
       </c>
       <c r="D21" s="6">
+        <v>38995</v>
+      </c>
+      <c r="E21" s="7">
+        <v>46316</v>
+      </c>
+      <c r="F21" s="8">
+        <v>1</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A22" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="19">
+        <v>3138903</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="6">
+        <v>40526</v>
+      </c>
+      <c r="E22" s="7">
+        <v>46316</v>
+      </c>
+      <c r="F22" s="8">
+        <v>1</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="19">
+        <v>2842290</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="6">
+        <v>36959</v>
+      </c>
+      <c r="E23" s="7">
+        <v>46316</v>
+      </c>
+      <c r="F23" s="8">
+        <v>1</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A24" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="19">
+        <v>3161275</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="6">
+        <v>32986</v>
+      </c>
+      <c r="E24" s="7">
+        <v>46316</v>
+      </c>
+      <c r="F24" s="8">
+        <v>1</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="19">
+        <v>3133871</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25" s="6">
         <v>20622</v>
       </c>
-      <c r="E21" s="7">
-        <v>46279</v>
-      </c>
-      <c r="F21" s="8">
-        <v>0</v>
-      </c>
-      <c r="G21" s="6" t="s">
+      <c r="E25" s="7">
+        <v>46316</v>
+      </c>
+      <c r="F25" s="8">
+        <v>1</v>
+      </c>
+      <c r="G25" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A22" s="21" t="s">
+    <row r="26" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A26" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="19">
+        <v>2546120</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="6">
+        <v>30172</v>
+      </c>
+      <c r="E26" s="7">
+        <v>46317</v>
+      </c>
+      <c r="F26" s="8">
+        <v>1</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A27" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="19">
+        <v>3483885</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="6">
+        <v>30172</v>
+      </c>
+      <c r="E27" s="7">
+        <v>46317</v>
+      </c>
+      <c r="F27" s="8">
+        <v>1</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A28" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="19">
+        <v>2460499</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="6">
+        <v>40438</v>
+      </c>
+      <c r="E28" s="7">
+        <v>46317</v>
+      </c>
+      <c r="F28" s="8">
+        <v>1</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A29" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="19">
+        <v>2621989</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="6">
+        <v>40438</v>
+      </c>
+      <c r="E29" s="7">
+        <v>46317</v>
+      </c>
+      <c r="F29" s="8">
+        <v>1</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A30" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="19">
+        <v>2556156</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D30" s="6">
+        <v>40437</v>
+      </c>
+      <c r="E30" s="7">
+        <v>46317</v>
+      </c>
+      <c r="F30" s="8">
+        <v>1</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A31" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="20">
+      <c r="B31" s="19">
         <v>4927976</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C31" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D31" s="6">
         <v>40437</v>
       </c>
-      <c r="E22" s="7">
-        <v>46275</v>
-      </c>
-      <c r="F22" s="8">
-        <v>0</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A23" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="B23" s="20">
-        <v>3133871</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="D23" s="6">
-        <v>20622</v>
-      </c>
-      <c r="E23" s="7">
-        <v>46279</v>
-      </c>
-      <c r="F23" s="8">
-        <v>0</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A24" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" s="20">
-        <v>2469229</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="D24" s="6">
-        <v>25212</v>
-      </c>
-      <c r="E24" s="7">
-        <v>46267</v>
-      </c>
-      <c r="F24" s="8">
-        <v>0</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A25" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="B25" s="20">
-        <v>5257024</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25" s="6">
-        <v>29911</v>
-      </c>
-      <c r="E25" s="7">
-        <v>46267</v>
-      </c>
-      <c r="F25" s="8">
-        <v>0</v>
-      </c>
-      <c r="G25" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A26" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="B26" s="20">
-        <v>4232277</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="D26" s="6">
-        <v>38977</v>
-      </c>
-      <c r="E26" s="7">
-        <v>46275</v>
-      </c>
-      <c r="F26" s="8">
-        <v>0</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A27" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="B27" s="24">
-        <v>2842290</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" s="25">
-        <v>36959</v>
-      </c>
-      <c r="E27" s="26">
-        <v>46287</v>
-      </c>
-      <c r="F27" s="27">
-        <v>0</v>
-      </c>
-      <c r="G27" s="25" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A28" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="B28" s="20">
-        <v>3161275</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" s="6">
-        <v>32986</v>
-      </c>
-      <c r="E28" s="7">
-        <v>46287</v>
-      </c>
-      <c r="F28" s="8">
-        <v>0</v>
-      </c>
-      <c r="G28" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A29" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" s="20">
-        <v>2676088</v>
-      </c>
-      <c r="C29" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" s="6">
-        <v>29905</v>
-      </c>
-      <c r="E29" s="7">
-        <v>46267</v>
-      </c>
-      <c r="F29" s="8">
-        <v>0</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="36" x14ac:dyDescent="0.25">
-      <c r="A30" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="20">
-        <v>3480805</v>
-      </c>
-      <c r="C30" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="D30" s="6">
-        <v>41517</v>
-      </c>
-      <c r="E30" s="7">
-        <v>46267</v>
-      </c>
-      <c r="F30" s="8">
-        <v>0</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A31" s="23" t="s">
+      <c r="E31" s="7">
+        <v>46317</v>
+      </c>
+      <c r="F31" s="8">
+        <v>1</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A32" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="B31" s="20">
+      <c r="B32" s="19">
         <v>3277548</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="C32" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D31" s="25">
+      <c r="D32" s="6">
         <v>40437</v>
       </c>
-      <c r="E31" s="26">
-        <v>46275</v>
-      </c>
-      <c r="F31" s="27">
-        <v>1</v>
-      </c>
-      <c r="G31" s="25" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="24" x14ac:dyDescent="0.25">
-      <c r="A32" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="B32" s="20">
-        <v>2553990</v>
-      </c>
-      <c r="C32" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="D32" s="6">
-        <v>29116</v>
-      </c>
       <c r="E32" s="7">
-        <v>46275</v>
+        <v>46317</v>
       </c>
       <c r="F32" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="24" x14ac:dyDescent="0.25">
-      <c r="A33" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="B33" s="20">
-        <v>4762128</v>
-      </c>
-      <c r="C33" s="19" t="s">
+      <c r="A33" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" s="19">
+        <v>3741720</v>
+      </c>
+      <c r="C33" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D33" s="6">
         <v>28209</v>
       </c>
       <c r="E33" s="7">
-        <v>46279</v>
+        <v>46317</v>
       </c>
       <c r="F33" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A34" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="B34" s="20">
-        <v>5257066</v>
+    <row r="34" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A34" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B34" s="19">
+        <v>5256354</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D34" s="6">
-        <v>38700</v>
+        <v>28209</v>
       </c>
       <c r="E34" s="7">
-        <v>46274</v>
+        <v>46317</v>
       </c>
       <c r="F34" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A35" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="B35" s="20">
-        <v>2686533</v>
+      <c r="A35" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="19">
+        <v>2676088</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D35" s="6">
-        <v>38977</v>
+        <v>29905</v>
       </c>
       <c r="E35" s="7">
-        <v>46275</v>
+        <v>46324</v>
       </c>
       <c r="F35" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="B36" s="20">
-        <v>2465181</v>
+    <row r="36" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A36" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" s="19">
+        <v>5257044</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D36" s="6">
-        <v>34238</v>
+        <v>28209</v>
       </c>
       <c r="E36" s="7">
-        <v>46267</v>
+        <v>46324</v>
       </c>
       <c r="F36" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A37" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="B37" s="20">
-        <v>3499270</v>
+    <row r="37" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A37" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" s="19">
+        <v>4762128</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D37" s="6">
-        <v>38977</v>
+        <v>28209</v>
       </c>
       <c r="E37" s="7">
-        <v>46275</v>
+        <v>46324</v>
       </c>
       <c r="F37" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A38" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="B38" s="20">
-        <v>3483855</v>
-      </c>
-      <c r="C38" s="19" t="s">
-        <v>9</v>
+    <row r="38" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A38" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38" s="19">
+        <v>3582671</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>66</v>
       </c>
       <c r="D38" s="6">
-        <v>38995</v>
-      </c>
-      <c r="E38" s="7"/>
+        <v>27575</v>
+      </c>
+      <c r="E38" s="7">
+        <v>46324</v>
+      </c>
       <c r="F38" s="8">
-        <v>0</v>
-      </c>
-      <c r="G38" s="6" t="s">
-        <v>8</v>
+        <v>1</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A39" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="B39" s="20">
-        <v>2621989</v>
-      </c>
-      <c r="C39" s="19" t="s">
-        <v>19</v>
+      <c r="A39" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39" s="19">
+        <v>5257024</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>25</v>
       </c>
       <c r="D39" s="6">
-        <v>40438</v>
+        <v>29911</v>
       </c>
       <c r="E39" s="7">
-        <v>46287</v>
+        <v>46324</v>
       </c>
       <c r="F39" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A40" s="15"/>
+      <c r="A40" s="14"/>
       <c r="B40" s="6"/>
-      <c r="C40" s="17"/>
+      <c r="C40" s="16"/>
       <c r="D40" s="6"/>
       <c r="E40" s="7"/>
       <c r="F40" s="8"/>
       <c r="G40" s="6"/>
     </row>
     <row r="41" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A41" s="16"/>
+      <c r="A41" s="15"/>
       <c r="B41" s="6"/>
-      <c r="C41" s="17"/>
+      <c r="C41" s="16"/>
       <c r="D41" s="6"/>
       <c r="E41" s="7"/>
       <c r="F41" s="8"/>
@@ -1680,7 +1639,7 @@
     <row r="42" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
       <c r="B42" s="6"/>
-      <c r="C42" s="17"/>
+      <c r="C42" s="16"/>
       <c r="D42" s="6"/>
       <c r="E42" s="7"/>
       <c r="F42" s="8"/>
@@ -1700,7 +1659,7 @@
   </sheetData>
   <autoFilter ref="A1:G43" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G43">
-      <sortCondition ref="A1:A43"/>
+      <sortCondition ref="E1:E43"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>